<commit_message>
PRL-MRP-007: create governed signal inventory workbook tab
</commit_message>
<xml_diff>
--- a/data/reference/signal_workbooks/2026-03-25_NVDA_SIGNAL_WORKBOOK_v3_bounds_handoff_copy.xlsx
+++ b/data/reference/signal_workbooks/2026-03-25_NVDA_SIGNAL_WORKBOOK_v3_bounds_handoff_copy.xlsx
@@ -2,33 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re0fd4e4d6f344391"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="2" r:id="Rb295738c8a38442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Packs" sheetId="3" r:id="Rc2c32886dddf4f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Catalog" sheetId="4" r:id="R52123986d1394cf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anchor_Data" sheetId="5" r:id="R12ac3dcb11f84941"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live_Web_Baseline" sheetId="6" r:id="Ra0ff0a303dd04d6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthetic_Raw" sheetId="7" r:id="Re7e406ea50264482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Beta_Leadership" sheetId="8" r:id="R718b3f5f76564b54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Vol_Rates_FX" sheetId="9" r:id="R33c87539cfb548c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Execution_Options" sheetId="10" r:id="R9b9c5ecbe02f47ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Asia_Breadth" sheetId="11" r:id="Raa1972ed46154f84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Use_Cases" sheetId="12" r:id="R34a9e47eb30e40a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal_Step1_Framework" sheetId="13" r:id="Rcf421c4b82f84db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal_Step1_Tests" sheetId="14" r:id="Rbff71e5975254a7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Primitives_Catalog" sheetId="15" r:id="R7cda482ac64b44d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Features_Catalog" sheetId="16" r:id="Rfc90758b481646e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options_Chain_Raw_Spec" sheetId="17" r:id="R4ce9f16255b74c58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volume_Baseline_Raw_Spec" sheetId="18" r:id="R5d7a3030b7244be7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Playbook_Module_Audit" sheetId="19" r:id="R9d080c253a0f47e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate_41_44_Summary" sheetId="20" r:id="Re875af675e6d4f8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Python_Inventory" sheetId="21" r:id="Re398cf9ba6ed42d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Stage_Summary" sheetId="22" r:id="R1d9786c597c34a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Surface_Drivers" sheetId="23" r:id="Redce11407a644250"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coeff_Universe_Index" sheetId="24" r:id="R0fa89b289bff4c9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bounds_Method" sheetId="25" r:id="Rfe7d481aabca4a38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal_Bounds_Draft" sheetId="26" r:id="Ra8a7c143afbc40c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signal_Coeff_Handoff" sheetId="27" r:id="Rf0eafcb8e8bd4333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb042c5fdca2444d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="2" r:id="R31a2710b3928498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Packs" sheetId="3" r:id="R27bd425f08074ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Catalog" sheetId="4" r:id="R3f130b47626c4121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anchor_Data" sheetId="5" r:id="R594cfe323dab4a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live_Web_Baseline" sheetId="6" r:id="Rc107bf8a5fbf4a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthetic_Raw" sheetId="7" r:id="R76e1676567dd4f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Beta_Leadership" sheetId="8" r:id="R082c51a3795a4712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Vol_Rates_FX" sheetId="9" r:id="R8aca34ea08a4416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Execution_Options" sheetId="10" r:id="R733d35827044432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Asia_Breadth" sheetId="11" r:id="R682bf9dd552d4e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Use_Cases" sheetId="12" r:id="Rb739e45a3c2746fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal_Step1_Framework" sheetId="13" r:id="R163fef75c8df43ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal_Step1_Tests" sheetId="14" r:id="R0eaf0f3f240e44ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Primitives_Catalog" sheetId="15" r:id="Rf7a5948060bd43cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived_Features_Catalog" sheetId="16" r:id="Ra2be6fc92f4c4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options_Chain_Raw_Spec" sheetId="17" r:id="Rb3e6557e91d1436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volume_Baseline_Raw_Spec" sheetId="18" r:id="R0df0eb57a72e4e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Playbook_Module_Audit" sheetId="19" r:id="R2dea47124c934d50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate_41_44_Summary" sheetId="20" r:id="Rbc4442000c074182"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Python_Inventory" sheetId="21" r:id="R2ddf095ae8834da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Stage_Summary" sheetId="22" r:id="R3c3f468e958f45e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Surface_Drivers" sheetId="23" r:id="R9386b50c44014587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coeff_Universe_Index" sheetId="24" r:id="Rf877bcf1275d418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bounds_Method" sheetId="25" r:id="Rfdea4bbea2d847f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal_Bounds_Draft" sheetId="26" r:id="R94133b04509f4fa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signal_Coeff_Handoff" sheetId="27" r:id="R467bb2d3504b417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parallel Risk Lane Signal Inventory" sheetId="28" r:id="Rb3bb02e8717d42da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -416,7 +417,7 @@
     <x:numFmt numFmtId="167" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <x:numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -480,8 +481,20 @@
       <x:color theme="1"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -531,6 +544,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor theme="5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="1F4E78"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -601,7 +619,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="104">
+  <x:cellXfs count="167">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="left"/>
@@ -865,6 +883,161 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="166" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="166" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="2" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="2" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1446,7 +1619,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra13207660c3c4056"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R102d08096a094faa"/>
 </x:worksheet>
 </file>
 
@@ -2196,7 +2369,7 @@
     <x:mergeCell ref="A1:M1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R142851c850524dff"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa3ddaf0b394105"/>
 </x:worksheet>
 </file>
 
@@ -5224,7 +5397,7 @@
     <x:mergeCell ref="A65:L65"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21ef8e175c4344c0"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68b3825fe1c34dd1"/>
 </x:worksheet>
 </file>
 
@@ -11561,7 +11734,7 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04bba997810c4dc6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b51879ecdbb4d5a"/>
 </x:worksheet>
 </file>
 
@@ -21894,6 +22067,1268 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
   </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="34" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="163" t="str">
+        <x:v>Parallel Risk Lane Signal Inventory</x:v>
+      </x:c>
+      <x:c r="B1" s="163" t="str"/>
+      <x:c r="C1" s="163" t="str"/>
+      <x:c r="D1" s="163" t="str"/>
+      <x:c r="E1" s="163" t="str"/>
+      <x:c r="F1" s="163" t="str"/>
+      <x:c r="G1" s="163" t="str"/>
+      <x:c r="H1" s="163" t="str"/>
+      <x:c r="I1" s="163" t="str"/>
+      <x:c r="J1" s="163" t="str"/>
+      <x:c r="K1" s="163" t="str"/>
+      <x:c r="L1" s="163" t="str"/>
+      <x:c r="M1" s="163" t="str"/>
+      <x:c r="N1" s="163" t="str"/>
+      <x:c r="O1" s="163" t="str"/>
+      <x:c r="P1" s="163" t="str"/>
+      <x:c r="Q1" s="163" t="str"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Governed workbook reference tab. Runtime PRL must consume typed promotion artefacts only; no direct workbook reads.</x:v>
+      </x:c>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+      <x:c r="G2" t="str"/>
+      <x:c r="H2" t="str"/>
+      <x:c r="I2" t="str"/>
+      <x:c r="J2" t="str"/>
+      <x:c r="K2" t="str"/>
+      <x:c r="L2" t="str"/>
+      <x:c r="M2" t="str"/>
+      <x:c r="N2" t="str"/>
+      <x:c r="O2" t="str"/>
+      <x:c r="P2" t="str"/>
+      <x:c r="Q2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="166" t="str">
+        <x:v>signal_id</x:v>
+      </x:c>
+      <x:c r="B3" s="166" t="str">
+        <x:v>signal_family</x:v>
+      </x:c>
+      <x:c r="C3" s="166" t="str">
+        <x:v>inventory_status</x:v>
+      </x:c>
+      <x:c r="D3" s="166" t="str">
+        <x:v>raw_workbook_lineage_ref</x:v>
+      </x:c>
+      <x:c r="E3" s="166" t="str">
+        <x:v>derived_workbook_lineage_ref</x:v>
+      </x:c>
+      <x:c r="F3" s="166" t="str">
+        <x:v>runtime_contract_target</x:v>
+      </x:c>
+      <x:c r="G3" s="166" t="str">
+        <x:v>lawful_prl_use</x:v>
+      </x:c>
+      <x:c r="H3" s="166" t="str">
+        <x:v>runtime_use_permission</x:v>
+      </x:c>
+      <x:c r="I3" s="166" t="str">
+        <x:v>required_for_current_atom</x:v>
+      </x:c>
+      <x:c r="J3" s="166" t="str">
+        <x:v>raw_derived_config_trace_classification</x:v>
+      </x:c>
+      <x:c r="K3" s="166" t="str">
+        <x:v>missing_handling</x:v>
+      </x:c>
+      <x:c r="L3" s="166" t="str">
+        <x:v>unavailable_handling</x:v>
+      </x:c>
+      <x:c r="M3" s="166" t="str">
+        <x:v>exclusion_reason</x:v>
+      </x:c>
+      <x:c r="N3" s="166" t="str">
+        <x:v>status_rationale</x:v>
+      </x:c>
+      <x:c r="O3" s="166" t="str">
+        <x:v>risk_semantics_note</x:v>
+      </x:c>
+      <x:c r="P3" s="166" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+      <x:c r="Q3" s="166" t="str">
+        <x:v>promotion_record_key</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="87" t="str">
+        <x:v>source_time_utc</x:v>
+      </x:c>
+      <x:c r="B4" s="87" t="str">
+        <x:v>source_temporal</x:v>
+      </x:c>
+      <x:c r="C4" s="87" t="str">
+        <x:v>available_now</x:v>
+      </x:c>
+      <x:c r="D4" s="87" t="str">
+        <x:v>Raw_Primitives_Catalog!A3:H9</x:v>
+      </x:c>
+      <x:c r="E4" s="87" t="str"/>
+      <x:c r="F4" s="87" t="str">
+        <x:v>SignalSnapshotEntry</x:v>
+      </x:c>
+      <x:c r="G4" s="87" t="str">
+        <x:v>yes_after_typed_promotion</x:v>
+      </x:c>
+      <x:c r="H4" s="87" t="str">
+        <x:v>runtime_allowed_from_typed_inputs_only</x:v>
+      </x:c>
+      <x:c r="I4" s="87" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J4" s="87" t="str">
+        <x:v>metadata</x:v>
+      </x:c>
+      <x:c r="K4" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L4" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="M4" s="87" t="str"/>
+      <x:c r="N4" s="87" t="str">
+        <x:v>Temporal source time is already carried by typed TemporalContextInput.</x:v>
+      </x:c>
+      <x:c r="O4" s="87" t="str">
+        <x:v>neutral state-of-play timing metadata</x:v>
+      </x:c>
+      <x:c r="P4" s="87" t="str">
+        <x:v>No direct workbook runtime read.</x:v>
+      </x:c>
+      <x:c r="Q4" s="87" t="str">
+        <x:v>source_time_utc</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="87" t="str">
+        <x:v>scheduled_event_window_active</x:v>
+      </x:c>
+      <x:c r="B5" s="87" t="str">
+        <x:v>calendar_event</x:v>
+      </x:c>
+      <x:c r="C5" s="87" t="str">
+        <x:v>available_now</x:v>
+      </x:c>
+      <x:c r="D5" s="87" t="str">
+        <x:v>Raw_Primitives_Catalog!A3:H9</x:v>
+      </x:c>
+      <x:c r="E5" s="87" t="str"/>
+      <x:c r="F5" s="87" t="str">
+        <x:v>EventProximityRegisterEntry</x:v>
+      </x:c>
+      <x:c r="G5" s="87" t="str">
+        <x:v>yes_after_typed_promotion</x:v>
+      </x:c>
+      <x:c r="H5" s="87" t="str">
+        <x:v>runtime_allowed_from_typed_inputs_only</x:v>
+      </x:c>
+      <x:c r="I5" s="87" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J5" s="87" t="str">
+        <x:v>metadata</x:v>
+      </x:c>
+      <x:c r="K5" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L5" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="M5" s="87" t="str"/>
+      <x:c r="N5" s="87" t="str">
+        <x:v>Scheduled event windows are typed temporal inputs.</x:v>
+      </x:c>
+      <x:c r="O5" s="87" t="str">
+        <x:v>event proximity may be constructive, defensive, mixed, or uncertain</x:v>
+      </x:c>
+      <x:c r="P5" s="87" t="str">
+        <x:v>No trade action authority.</x:v>
+      </x:c>
+      <x:c r="Q5" s="87" t="str">
+        <x:v>scheduled_event_window_active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="87" t="str">
+        <x:v>vix_level</x:v>
+      </x:c>
+      <x:c r="B6" s="87" t="str">
+        <x:v>market_volatility_context</x:v>
+      </x:c>
+      <x:c r="C6" s="87" t="str">
+        <x:v>available_now</x:v>
+      </x:c>
+      <x:c r="D6" s="87" t="str">
+        <x:v>Runtime_Surface_Drivers!A4:K9</x:v>
+      </x:c>
+      <x:c r="E6" s="87" t="str">
+        <x:v>Coeff_Universe_Index!A4:L9</x:v>
+      </x:c>
+      <x:c r="F6" s="87" t="str">
+        <x:v>SignalSnapshotEntry</x:v>
+      </x:c>
+      <x:c r="G6" s="87" t="str">
+        <x:v>yes_after_typed_promotion</x:v>
+      </x:c>
+      <x:c r="H6" s="87" t="str">
+        <x:v>runtime_allowed_from_typed_inputs_only</x:v>
+      </x:c>
+      <x:c r="I6" s="87" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J6" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K6" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L6" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="M6" s="87" t="str"/>
+      <x:c r="N6" s="87" t="str">
+        <x:v>VIX level is already represented on the typed regime input.</x:v>
+      </x:c>
+      <x:c r="O6" s="87" t="str">
+        <x:v>volatility terrain metadata, not a direction call</x:v>
+      </x:c>
+      <x:c r="P6" s="87" t="str">
+        <x:v>Compatibility thresholds remain governed separately.</x:v>
+      </x:c>
+      <x:c r="Q6" s="87" t="str">
+        <x:v>vix_level</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="87" t="str">
+        <x:v>spot_price</x:v>
+      </x:c>
+      <x:c r="B7" s="87" t="str">
+        <x:v>options_flow</x:v>
+      </x:c>
+      <x:c r="C7" s="87" t="str">
+        <x:v>available_now</x:v>
+      </x:c>
+      <x:c r="D7" s="87" t="str">
+        <x:v>Raw_Primitives_Catalog!A9:H18</x:v>
+      </x:c>
+      <x:c r="E7" s="87" t="str"/>
+      <x:c r="F7" s="87" t="str">
+        <x:v>SignalSnapshotEntry</x:v>
+      </x:c>
+      <x:c r="G7" s="87" t="str">
+        <x:v>yes_after_typed_promotion</x:v>
+      </x:c>
+      <x:c r="H7" s="87" t="str">
+        <x:v>runtime_allowed_from_typed_inputs_only</x:v>
+      </x:c>
+      <x:c r="I7" s="87" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J7" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K7" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L7" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="M7" s="87" t="str"/>
+      <x:c r="N7" s="87" t="str">
+        <x:v>Spot/underlying price is a typed options-flow primitive when present.</x:v>
+      </x:c>
+      <x:c r="O7" s="87" t="str">
+        <x:v>current market-state metadata</x:v>
+      </x:c>
+      <x:c r="P7" s="87" t="str">
+        <x:v>No order or sizing authority.</x:v>
+      </x:c>
+      <x:c r="Q7" s="87" t="str">
+        <x:v>spot_price</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="87" t="str">
+        <x:v>front_dte</x:v>
+      </x:c>
+      <x:c r="B8" s="87" t="str">
+        <x:v>options_repricing_context</x:v>
+      </x:c>
+      <x:c r="C8" s="87" t="str">
+        <x:v>available_now</x:v>
+      </x:c>
+      <x:c r="D8" s="87" t="str">
+        <x:v>Raw_Primitives_Catalog!A7:H8</x:v>
+      </x:c>
+      <x:c r="E8" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="F8" s="87" t="str">
+        <x:v>SignalSnapshotEntry</x:v>
+      </x:c>
+      <x:c r="G8" s="87" t="str">
+        <x:v>yes_after_typed_promotion</x:v>
+      </x:c>
+      <x:c r="H8" s="87" t="str">
+        <x:v>runtime_allowed_from_typed_inputs_only</x:v>
+      </x:c>
+      <x:c r="I8" s="87" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J8" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K8" s="87" t="str">
+        <x:v>disables_atom_if_missing</x:v>
+      </x:c>
+      <x:c r="L8" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="M8" s="87" t="str"/>
+      <x:c r="N8" s="87" t="str">
+        <x:v>Front DTE supports the existing options repricing atom.</x:v>
+      </x:c>
+      <x:c r="O8" s="87" t="str">
+        <x:v>options calendar state-of-play</x:v>
+      </x:c>
+      <x:c r="P8" s="87" t="str">
+        <x:v>No options strategy recommendation.</x:v>
+      </x:c>
+      <x:c r="Q8" s="87" t="str">
+        <x:v>front_dte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="87" t="str">
+        <x:v>next_dte</x:v>
+      </x:c>
+      <x:c r="B9" s="87" t="str">
+        <x:v>options_repricing_context</x:v>
+      </x:c>
+      <x:c r="C9" s="87" t="str">
+        <x:v>available_now</x:v>
+      </x:c>
+      <x:c r="D9" s="87" t="str">
+        <x:v>Raw_Primitives_Catalog!A7:H8</x:v>
+      </x:c>
+      <x:c r="E9" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="F9" s="87" t="str">
+        <x:v>SignalSnapshotEntry</x:v>
+      </x:c>
+      <x:c r="G9" s="87" t="str">
+        <x:v>yes_after_typed_promotion</x:v>
+      </x:c>
+      <x:c r="H9" s="87" t="str">
+        <x:v>runtime_allowed_from_typed_inputs_only</x:v>
+      </x:c>
+      <x:c r="I9" s="87" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J9" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K9" s="87" t="str">
+        <x:v>disables_atom_if_missing</x:v>
+      </x:c>
+      <x:c r="L9" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="M9" s="87" t="str"/>
+      <x:c r="N9" s="87" t="str">
+        <x:v>Next DTE supports the existing options repricing atom.</x:v>
+      </x:c>
+      <x:c r="O9" s="87" t="str">
+        <x:v>options calendar state-of-play</x:v>
+      </x:c>
+      <x:c r="P9" s="87" t="str">
+        <x:v>No options strategy recommendation.</x:v>
+      </x:c>
+      <x:c r="Q9" s="87" t="str">
+        <x:v>next_dte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="87" t="str">
+        <x:v>regime_context_packet</x:v>
+      </x:c>
+      <x:c r="B10" s="87" t="str">
+        <x:v>macro_regime</x:v>
+      </x:c>
+      <x:c r="C10" s="87" t="str">
+        <x:v>upstream_but_not_projected</x:v>
+      </x:c>
+      <x:c r="D10" s="87" t="str">
+        <x:v>Runtime_Surface_Drivers!A4:K12</x:v>
+      </x:c>
+      <x:c r="E10" s="87" t="str"/>
+      <x:c r="F10" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G10" s="87" t="str">
+        <x:v>no_until_projection_admitted</x:v>
+      </x:c>
+      <x:c r="H10" s="87" t="str">
+        <x:v>not_runtime_allowed_until_typed_projection</x:v>
+      </x:c>
+      <x:c r="I10" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J10" s="87" t="str">
+        <x:v>trace</x:v>
+      </x:c>
+      <x:c r="K10" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L10" s="87" t="str">
+        <x:v>unavailable_register_entry</x:v>
+      </x:c>
+      <x:c r="M10" s="87" t="str"/>
+      <x:c r="N10" s="87" t="str">
+        <x:v>Regime primitives exist but only selected fields are admitted to the current PRL.</x:v>
+      </x:c>
+      <x:c r="O10" s="87" t="str">
+        <x:v>macro regime context metadata</x:v>
+      </x:c>
+      <x:c r="P10" s="87" t="str">
+        <x:v>Future projection must remain typed.</x:v>
+      </x:c>
+      <x:c r="Q10" s="87" t="str">
+        <x:v>regime_context_packet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="87" t="str">
+        <x:v>options_flow_context_packet</x:v>
+      </x:c>
+      <x:c r="B11" s="87" t="str">
+        <x:v>options_flow</x:v>
+      </x:c>
+      <x:c r="C11" s="87" t="str">
+        <x:v>upstream_but_not_projected</x:v>
+      </x:c>
+      <x:c r="D11" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="E11" s="87" t="str"/>
+      <x:c r="F11" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G11" s="87" t="str">
+        <x:v>no_until_projection_admitted</x:v>
+      </x:c>
+      <x:c r="H11" s="87" t="str">
+        <x:v>not_runtime_allowed_until_typed_projection</x:v>
+      </x:c>
+      <x:c r="I11" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J11" s="87" t="str">
+        <x:v>trace</x:v>
+      </x:c>
+      <x:c r="K11" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L11" s="87" t="str">
+        <x:v>unavailable_register_entry</x:v>
+      </x:c>
+      <x:c r="M11" s="87" t="str"/>
+      <x:c r="N11" s="87" t="str">
+        <x:v>Options-flow packet exists as upstream context but rich chain fields are not admitted.</x:v>
+      </x:c>
+      <x:c r="O11" s="87" t="str">
+        <x:v>options-flow state metadata</x:v>
+      </x:c>
+      <x:c r="P11" s="87" t="str">
+        <x:v>No fabricated chain values.</x:v>
+      </x:c>
+      <x:c r="Q11" s="87" t="str">
+        <x:v>options_flow_context_packet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="87" t="str">
+        <x:v>distance_to_vwap</x:v>
+      </x:c>
+      <x:c r="B12" s="87" t="str">
+        <x:v>market_microstructure</x:v>
+      </x:c>
+      <x:c r="C12" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D12" s="87" t="str">
+        <x:v>Raw_Primitives_Catalog!A9:H24</x:v>
+      </x:c>
+      <x:c r="E12" s="87" t="str">
+        <x:v>Derived_Features_Catalog!A3:H6</x:v>
+      </x:c>
+      <x:c r="F12" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G12" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H12" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I12" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J12" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K12" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L12" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M12" s="87" t="str"/>
+      <x:c r="N12" s="87" t="str">
+        <x:v>VWAP distance lacks a typed PRL runtime source.</x:v>
+      </x:c>
+      <x:c r="O12" s="87" t="str">
+        <x:v>microstructure terrain can be constructive or fragile</x:v>
+      </x:c>
+      <x:c r="P12" s="87" t="str">
+        <x:v>Deferred; no fabricated VWAP.</x:v>
+      </x:c>
+      <x:c r="Q12" s="87" t="str">
+        <x:v>distance_to_vwap</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="87" t="str">
+        <x:v>bid_ask_spread</x:v>
+      </x:c>
+      <x:c r="B13" s="87" t="str">
+        <x:v>liquidity_depth</x:v>
+      </x:c>
+      <x:c r="C13" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D13" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="E13" s="87" t="str"/>
+      <x:c r="F13" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G13" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H13" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I13" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J13" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K13" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L13" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M13" s="87" t="str"/>
+      <x:c r="N13" s="87" t="str">
+        <x:v>NBBO/depth source is not typed for current PRL.</x:v>
+      </x:c>
+      <x:c r="O13" s="87" t="str">
+        <x:v>liquidity state metadata</x:v>
+      </x:c>
+      <x:c r="P13" s="87" t="str">
+        <x:v>Deferred; no fabricated spread/depth.</x:v>
+      </x:c>
+      <x:c r="Q13" s="87" t="str">
+        <x:v>bid_ask_spread</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="87" t="str">
+        <x:v>tape_speed_relative_volume</x:v>
+      </x:c>
+      <x:c r="B14" s="87" t="str">
+        <x:v>activity_legibility</x:v>
+      </x:c>
+      <x:c r="C14" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D14" s="87" t="str">
+        <x:v>Volume_Baseline_Raw_Spec!A1:H9</x:v>
+      </x:c>
+      <x:c r="E14" s="87" t="str">
+        <x:v>Derived_Features_Catalog!A3:H12</x:v>
+      </x:c>
+      <x:c r="F14" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G14" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H14" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I14" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J14" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K14" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L14" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M14" s="87" t="str"/>
+      <x:c r="N14" s="87" t="str">
+        <x:v>Volume curve/tape speed is not typed for current PRL.</x:v>
+      </x:c>
+      <x:c r="O14" s="87" t="str">
+        <x:v>activity legibility metadata</x:v>
+      </x:c>
+      <x:c r="P14" s="87" t="str">
+        <x:v>Deferred; no fabricated relative volume.</x:v>
+      </x:c>
+      <x:c r="Q14" s="87" t="str">
+        <x:v>tape_speed_relative_volume</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="87" t="str">
+        <x:v>realised_volatility_atr</x:v>
+      </x:c>
+      <x:c r="B15" s="87" t="str">
+        <x:v>range_state</x:v>
+      </x:c>
+      <x:c r="C15" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D15" s="87" t="str">
+        <x:v>Raw_Primitives_Catalog!A9:H24</x:v>
+      </x:c>
+      <x:c r="E15" s="87" t="str">
+        <x:v>Derived_Features_Catalog!A7:H12</x:v>
+      </x:c>
+      <x:c r="F15" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G15" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H15" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I15" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J15" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K15" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L15" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M15" s="87" t="str"/>
+      <x:c r="N15" s="87" t="str">
+        <x:v>Realised volatility/ATR requires typed bar-series source.</x:v>
+      </x:c>
+      <x:c r="O15" s="87" t="str">
+        <x:v>range and disorder state metadata</x:v>
+      </x:c>
+      <x:c r="P15" s="87" t="str">
+        <x:v>Deferred; no fabricated ATR.</x:v>
+      </x:c>
+      <x:c r="Q15" s="87" t="str">
+        <x:v>realised_volatility_atr</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="87" t="str">
+        <x:v>dense_options_chain</x:v>
+      </x:c>
+      <x:c r="B16" s="87" t="str">
+        <x:v>options_surface</x:v>
+      </x:c>
+      <x:c r="C16" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D16" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="E16" s="87" t="str"/>
+      <x:c r="F16" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G16" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H16" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I16" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J16" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K16" s="87" t="str">
+        <x:v>disables_atom_if_missing</x:v>
+      </x:c>
+      <x:c r="L16" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M16" s="87" t="str"/>
+      <x:c r="N16" s="87" t="str">
+        <x:v>Dense options chain is not a current typed PRL input.</x:v>
+      </x:c>
+      <x:c r="O16" s="87" t="str">
+        <x:v>options-surface availability metadata</x:v>
+      </x:c>
+      <x:c r="P16" s="87" t="str">
+        <x:v>Deferred; no fabricated chain state without lawful source.</x:v>
+      </x:c>
+      <x:c r="Q16" s="87" t="str">
+        <x:v>dense_options_chain</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="87" t="str">
+        <x:v>iv_rank_implied_move</x:v>
+      </x:c>
+      <x:c r="B17" s="87" t="str">
+        <x:v>event_volatility</x:v>
+      </x:c>
+      <x:c r="C17" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D17" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="E17" s="87" t="str">
+        <x:v>Derived_Execution_Options!A1:M15</x:v>
+      </x:c>
+      <x:c r="F17" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G17" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H17" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I17" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J17" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K17" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L17" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M17" s="87" t="str"/>
+      <x:c r="N17" s="87" t="str">
+        <x:v>IV rank/implied move requires typed options-vol context.</x:v>
+      </x:c>
+      <x:c r="O17" s="87" t="str">
+        <x:v>event-volatility state metadata</x:v>
+      </x:c>
+      <x:c r="P17" s="87" t="str">
+        <x:v>Deferred; no fabricated IV rank.</x:v>
+      </x:c>
+      <x:c r="Q17" s="87" t="str">
+        <x:v>iv_rank_implied_move</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="87" t="str">
+        <x:v>skew_state</x:v>
+      </x:c>
+      <x:c r="B18" s="87" t="str">
+        <x:v>options_skew</x:v>
+      </x:c>
+      <x:c r="C18" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D18" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="E18" s="87" t="str">
+        <x:v>Derived_Execution_Options!A1:M15</x:v>
+      </x:c>
+      <x:c r="F18" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G18" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H18" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I18" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J18" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K18" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L18" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M18" s="87" t="str"/>
+      <x:c r="N18" s="87" t="str">
+        <x:v>Skew requires typed strike/expiry IV surface.</x:v>
+      </x:c>
+      <x:c r="O18" s="87" t="str">
+        <x:v>asymmetry state metadata</x:v>
+      </x:c>
+      <x:c r="P18" s="87" t="str">
+        <x:v>Deferred; no fabricated skew.</x:v>
+      </x:c>
+      <x:c r="Q18" s="87" t="str">
+        <x:v>skew_state</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="87" t="str">
+        <x:v>gamma_exposure_flip</x:v>
+      </x:c>
+      <x:c r="B19" s="87" t="str">
+        <x:v>dealer_convexity</x:v>
+      </x:c>
+      <x:c r="C19" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D19" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="E19" s="87" t="str">
+        <x:v>Derived_Execution_Options!A1:M15</x:v>
+      </x:c>
+      <x:c r="F19" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G19" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H19" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I19" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J19" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K19" s="87" t="str">
+        <x:v>disables_atom_if_missing</x:v>
+      </x:c>
+      <x:c r="L19" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M19" s="87" t="str"/>
+      <x:c r="N19" s="87" t="str">
+        <x:v>Gamma exposure/gamma flip requires typed greeks/OI/spot model.</x:v>
+      </x:c>
+      <x:c r="O19" s="87" t="str">
+        <x:v>dealer-convexity state metadata</x:v>
+      </x:c>
+      <x:c r="P19" s="87" t="str">
+        <x:v>Deferred; no fabricated gamma.</x:v>
+      </x:c>
+      <x:c r="Q19" s="87" t="str">
+        <x:v>gamma_exposure_flip</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="87" t="str">
+        <x:v>oi_concentration_strike_pin</x:v>
+      </x:c>
+      <x:c r="B20" s="87" t="str">
+        <x:v>strike_concentration</x:v>
+      </x:c>
+      <x:c r="C20" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D20" s="87" t="str">
+        <x:v>Options_Chain_Raw_Spec!A1:H21</x:v>
+      </x:c>
+      <x:c r="E20" s="87" t="str">
+        <x:v>Derived_Execution_Options!A1:M15</x:v>
+      </x:c>
+      <x:c r="F20" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G20" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H20" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I20" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J20" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K20" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L20" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M20" s="87" t="str"/>
+      <x:c r="N20" s="87" t="str">
+        <x:v>OI concentration/strike pin requires typed OI by strike and spot distance.</x:v>
+      </x:c>
+      <x:c r="O20" s="87" t="str">
+        <x:v>pinning/concentration metadata</x:v>
+      </x:c>
+      <x:c r="P20" s="87" t="str">
+        <x:v>Deferred; no fabricated OI concentration.</x:v>
+      </x:c>
+      <x:c r="Q20" s="87" t="str">
+        <x:v>oi_concentration_strike_pin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="87" t="str">
+        <x:v>moc_close_auction_imbalance</x:v>
+      </x:c>
+      <x:c r="B21" s="87" t="str">
+        <x:v>auction_state</x:v>
+      </x:c>
+      <x:c r="C21" s="87" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="D21" s="87" t="str"/>
+      <x:c r="E21" s="87" t="str"/>
+      <x:c r="F21" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G21" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H21" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I21" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J21" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K21" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L21" s="87" t="str">
+        <x:v>missing_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M21" s="87" t="str"/>
+      <x:c r="N21" s="87" t="str">
+        <x:v>Auction imbalance source is not present in the workbook or current runtime.</x:v>
+      </x:c>
+      <x:c r="O21" s="87" t="str">
+        <x:v>auction-state metadata</x:v>
+      </x:c>
+      <x:c r="P21" s="87" t="str">
+        <x:v>Missing until lawful source exists.</x:v>
+      </x:c>
+      <x:c r="Q21" s="87" t="str">
+        <x:v>moc_close_auction_imbalance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="87" t="str">
+        <x:v>headline_risk_context</x:v>
+      </x:c>
+      <x:c r="B22" s="87" t="str">
+        <x:v>headline_risk</x:v>
+      </x:c>
+      <x:c r="C22" s="87" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="D22" s="87" t="str"/>
+      <x:c r="E22" s="87" t="str"/>
+      <x:c r="F22" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G22" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H22" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I22" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J22" s="87" t="str">
+        <x:v>raw</x:v>
+      </x:c>
+      <x:c r="K22" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L22" s="87" t="str">
+        <x:v>missing_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M22" s="87" t="str"/>
+      <x:c r="N22" s="87" t="str">
+        <x:v>Governed headline source is not present in current runtime.</x:v>
+      </x:c>
+      <x:c r="O22" s="87" t="str">
+        <x:v>information-lag/conflict metadata</x:v>
+      </x:c>
+      <x:c r="P22" s="87" t="str">
+        <x:v>Missing until lawful source exists.</x:v>
+      </x:c>
+      <x:c r="Q22" s="87" t="str">
+        <x:v>headline_risk_context</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="87" t="str">
+        <x:v>crowding_real_money_flow</x:v>
+      </x:c>
+      <x:c r="B23" s="87" t="str">
+        <x:v>flow_positioning</x:v>
+      </x:c>
+      <x:c r="C23" s="87" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="D23" s="87" t="str"/>
+      <x:c r="E23" s="87" t="str"/>
+      <x:c r="F23" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G23" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H23" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I23" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J23" s="87" t="str">
+        <x:v>derived</x:v>
+      </x:c>
+      <x:c r="K23" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L23" s="87" t="str">
+        <x:v>missing_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M23" s="87" t="str"/>
+      <x:c r="N23" s="87" t="str">
+        <x:v>Crowding/real-money flow source is not present in current runtime.</x:v>
+      </x:c>
+      <x:c r="O23" s="87" t="str">
+        <x:v>positioning-pressure metadata</x:v>
+      </x:c>
+      <x:c r="P23" s="87" t="str">
+        <x:v>Missing until lawful source exists.</x:v>
+      </x:c>
+      <x:c r="Q23" s="87" t="str">
+        <x:v>crowding_real_money_flow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="87" t="str">
+        <x:v>cognitive_load_attention_pressure</x:v>
+      </x:c>
+      <x:c r="B24" s="87" t="str">
+        <x:v>attention_load</x:v>
+      </x:c>
+      <x:c r="C24" s="87" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="D24" s="87" t="str"/>
+      <x:c r="E24" s="87" t="str"/>
+      <x:c r="F24" s="87" t="str">
+        <x:v>ParallelRiskExpectedSignalRecord</x:v>
+      </x:c>
+      <x:c r="G24" s="87" t="str">
+        <x:v>no_until_typed_source_exists</x:v>
+      </x:c>
+      <x:c r="H24" s="87" t="str">
+        <x:v>not_runtime_allowed</x:v>
+      </x:c>
+      <x:c r="I24" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J24" s="87" t="str">
+        <x:v>metadata</x:v>
+      </x:c>
+      <x:c r="K24" s="87" t="str">
+        <x:v>lowers_confidence_if_missing</x:v>
+      </x:c>
+      <x:c r="L24" s="87" t="str">
+        <x:v>deferred_unavailable_no_value</x:v>
+      </x:c>
+      <x:c r="M24" s="87" t="str"/>
+      <x:c r="N24" s="87" t="str">
+        <x:v>Operator/context attention load lacks a typed source.</x:v>
+      </x:c>
+      <x:c r="O24" s="87" t="str">
+        <x:v>cognitive-friction state metadata</x:v>
+      </x:c>
+      <x:c r="P24" s="87" t="str">
+        <x:v>Deferred; no fabricated cognitive-load judgement without lawful source.</x:v>
+      </x:c>
+      <x:c r="Q24" s="87" t="str">
+        <x:v>cognitive_load_attention_pressure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="87" t="str">
+        <x:v>capital_sizing_signal</x:v>
+      </x:c>
+      <x:c r="B25" s="87" t="str">
+        <x:v>forbidden_authority</x:v>
+      </x:c>
+      <x:c r="C25" s="87" t="str">
+        <x:v>excluded</x:v>
+      </x:c>
+      <x:c r="D25" s="87" t="str"/>
+      <x:c r="E25" s="87" t="str"/>
+      <x:c r="F25" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="G25" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="H25" s="87" t="str">
+        <x:v>excluded_from_prl_runtime</x:v>
+      </x:c>
+      <x:c r="I25" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J25" s="87" t="str">
+        <x:v>config</x:v>
+      </x:c>
+      <x:c r="K25" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="L25" s="87" t="str">
+        <x:v>excluded_signal_not_demanded</x:v>
+      </x:c>
+      <x:c r="M25" s="87" t="str">
+        <x:v>capital sizing is downstream authority</x:v>
+      </x:c>
+      <x:c r="N25" s="87" t="str">
+        <x:v>Capital sizing cannot be a PRL signal.</x:v>
+      </x:c>
+      <x:c r="O25" s="87" t="str">
+        <x:v>authority boundary metadata</x:v>
+      </x:c>
+      <x:c r="P25" s="87" t="str">
+        <x:v>Excluded from runtime demand.</x:v>
+      </x:c>
+      <x:c r="Q25" s="87" t="str">
+        <x:v>capital_sizing_signal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="87" t="str">
+        <x:v>order_instruction_signal</x:v>
+      </x:c>
+      <x:c r="B26" s="87" t="str">
+        <x:v>forbidden_authority</x:v>
+      </x:c>
+      <x:c r="C26" s="87" t="str">
+        <x:v>excluded</x:v>
+      </x:c>
+      <x:c r="D26" s="87" t="str"/>
+      <x:c r="E26" s="87" t="str"/>
+      <x:c r="F26" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="G26" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="H26" s="87" t="str">
+        <x:v>excluded_from_prl_runtime</x:v>
+      </x:c>
+      <x:c r="I26" s="87" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J26" s="87" t="str">
+        <x:v>config</x:v>
+      </x:c>
+      <x:c r="K26" s="87" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="L26" s="87" t="str">
+        <x:v>excluded_signal_not_demanded</x:v>
+      </x:c>
+      <x:c r="M26" s="87" t="str">
+        <x:v>broker/order authority is downstream</x:v>
+      </x:c>
+      <x:c r="N26" s="87" t="str">
+        <x:v>Order instruction cannot be a PRL signal.</x:v>
+      </x:c>
+      <x:c r="O26" s="87" t="str">
+        <x:v>authority boundary metadata</x:v>
+      </x:c>
+      <x:c r="P26" s="87" t="str">
+        <x:v>Excluded from runtime demand.</x:v>
+      </x:c>
+      <x:c r="Q26" s="87" t="str">
+        <x:v>order_instruction_signal</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -24522,7 +25957,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb2869b688e44a35"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree5718710b1141e9"/>
 </x:worksheet>
 </file>
 
@@ -25878,7 +27313,7 @@
     <x:mergeCell ref="A1:AC1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re09b4ced9a70408c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88b6cb46cc534eb9"/>
 </x:worksheet>
 </file>
 
@@ -28599,7 +30034,7 @@
     <x:mergeCell ref="A1:AC1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f96acf7c6944825"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2bcf3977824cfc"/>
 </x:worksheet>
 </file>
 

</xml_diff>